<commit_message>
fix: robust unit classifier + catch budget-integer badges (148 numbers reformatted)
- classify money as 'บาท' preceded by 'ล' (handles Thai combining-order; was matching inner บาท)
- catches badge totals (3,788,000.0000) and ลบ.-garble integers; excludes พันล้านบาท/ไร่/ครั้ง/ล้านคน
- 149 ล้านบาท -> 148 baked to 4 decimals, fit-to-box (no overlap); ~114 flagged for review
- final PDF: 72 pages, live-text=0, float+TH-001+numbers fixed

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/audit_reports/B2G_Numbers_Audit.xlsx
+++ b/output/audit_reports/B2G_Numbers_Audit.xlsx
@@ -913,32 +913,36 @@
       <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>788,000</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>788,000</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr">
+      <c r="D17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>788,000.0000</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>บ.  uA} 788,000 au งบประมาณ ผู| |</t>
         </is>
@@ -1177,160 +1181,180 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>584,300</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>584,300</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
+      <c r="D25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>584,300.0000</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>ดเก็บ 3,584,300 au.  หักลด 584,30</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B26" t="n">
+      <c r="B26" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>3,788,000</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>3,788,000</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
+      <c r="D26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>3,788,000.0000</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>G 2570  3,788,000 au.  ที่มา : กระท</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>3,584,300</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>3,584,300</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
+      <c r="D27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>3,584,300.0000</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>จัดเก็บ 3,584,300 au.  หักลด 584,30</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>788,000</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>788,000</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr">
+      <c r="D28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>788,000.0000</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>2570  3,788,000 au.  ที่มา : กระท</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>3,000,000</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>3,000,000</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
+      <c r="D29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>3,000,000.0000</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>ินกู้ , 3,000,000 au.  SINUS:N1@UNI</t>
         </is>
@@ -1481,32 +1505,36 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B34" t="n">
+      <c r="B34" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>155,880</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>155,880</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
+      <c r="D34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>155,880.0000</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>500 ลบ. 155,880 au.  REVENUE รายไ</t>
         </is>
@@ -1893,32 +1921,36 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B46" t="n">
+      <c r="B46" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>3,788,000</t>
         </is>
       </c>
-      <c r="D46" t="n">
-        <v>0</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>บาท (ต่อหน่วย)</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>3,788,000</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr">
+      <c r="D46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>3,788,000.0000</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>บประมาณ 3,788,000 ลส้านบาท  ๕รรพ SS</t>
         </is>
@@ -2501,7 +2533,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านราย)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3237,7 +3269,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3681,7 +3713,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -3713,7 +3745,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -3809,7 +3841,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -3841,7 +3873,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -3905,7 +3937,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -3969,7 +4001,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -4001,7 +4033,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -4097,7 +4129,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -4129,7 +4161,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -4161,7 +4193,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -4641,7 +4673,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านราย)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -4737,7 +4769,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านราย)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -6181,32 +6213,36 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" t="n">
+      <c r="A175" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B175" t="n">
+      <c r="B175" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="C175" t="inlineStr">
+      <c r="C175" s="2" t="inlineStr">
         <is>
           <t>1,503,088.8</t>
         </is>
       </c>
-      <c r="D175" t="n">
-        <v>1</v>
-      </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>1,503,088.8</t>
-        </is>
-      </c>
-      <c r="G175" t="inlineStr"/>
-      <c r="H175" t="inlineStr">
+      <c r="D175" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>1,503,088.8000</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
         <is>
           <t>ล       1,503,088.8 aun  ด้านเศรษฐกิจ</t>
         </is>
@@ -6457,64 +6493,72 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="n">
+      <c r="A183" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B183" t="n">
+      <c r="B183" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="C183" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>185,939.3</t>
         </is>
       </c>
-      <c r="D183" t="n">
-        <v>1</v>
-      </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F183" t="inlineStr">
-        <is>
-          <t>185,939.3</t>
-        </is>
-      </c>
-      <c r="G183" t="inlineStr"/>
-      <c r="H183" t="inlineStr">
+      <c r="D183" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>185,939.3000</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>185,939.3 au. ด้านการค้า “เ</t>
         </is>
       </c>
     </row>
     <row r="184">
-      <c r="A184" t="n">
+      <c r="A184" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B184" t="n">
+      <c r="B184" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="C184" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>11,264.1</t>
         </is>
       </c>
-      <c r="D184" t="n">
-        <v>1</v>
-      </c>
-      <c r="E184" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F184" t="inlineStr">
-        <is>
-          <t>11,264.1</t>
-        </is>
-      </c>
-      <c r="G184" t="inlineStr"/>
-      <c r="H184" t="inlineStr">
+      <c r="D184" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>11,264.1000</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>11,264.1 au.  ค้านการต่างป</t>
         </is>
@@ -6557,32 +6601,36 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" t="n">
+      <c r="A186" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B186" t="n">
+      <c r="B186" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="C186" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>436,287.9</t>
         </is>
       </c>
-      <c r="D186" t="n">
-        <v>1</v>
-      </c>
-      <c r="E186" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F186" t="inlineStr">
-        <is>
-          <t>436,287.9</t>
-        </is>
-      </c>
-      <c r="G186" t="inlineStr"/>
-      <c r="H186" t="inlineStr">
+      <c r="D186" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>436,287.9000</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>436,287.9 au.  สร้างโอกาสกา</t>
         </is>
@@ -6625,32 +6673,36 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" t="n">
+      <c r="A188" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B188" t="n">
+      <c r="B188" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="C188" t="inlineStr">
+      <c r="C188" s="2" t="inlineStr">
         <is>
           <t>1,117.6</t>
         </is>
       </c>
-      <c r="D188" t="n">
-        <v>1</v>
-      </c>
-      <c r="E188" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F188" t="inlineStr">
-        <is>
-          <t>1,117.6</t>
-        </is>
-      </c>
-      <c r="G188" t="inlineStr"/>
-      <c r="H188" t="inlineStr">
+      <c r="D188" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>1,117.6000</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
         <is>
           <t>1,117.6 au.  เสริมสร้างเส</t>
         </is>
@@ -6765,32 +6817,36 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" t="n">
+      <c r="A192" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B192" t="n">
+      <c r="B192" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="C192" t="inlineStr">
+      <c r="C192" s="2" t="inlineStr">
         <is>
           <t>2,114.5</t>
         </is>
       </c>
-      <c r="D192" t="n">
-        <v>1</v>
-      </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F192" t="inlineStr">
-        <is>
-          <t>2,114.5</t>
-        </is>
-      </c>
-      <c r="G192" t="inlineStr"/>
-      <c r="H192" t="inlineStr">
+      <c r="D192" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>2,114.5000</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
         <is>
           <t>2,114.5 au.  BUDGET BUREA</t>
         </is>
@@ -6977,32 +7033,36 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" t="n">
+      <c r="A198" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B198" t="n">
+      <c r="B198" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="C198" t="inlineStr">
+      <c r="C198" s="2" t="inlineStr">
         <is>
           <t>4,940.4</t>
         </is>
       </c>
-      <c r="D198" t="n">
-        <v>1</v>
-      </c>
-      <c r="E198" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F198" t="inlineStr">
-        <is>
-          <t>4,940.4</t>
-        </is>
-      </c>
-      <c r="G198" t="inlineStr"/>
-      <c r="H198" t="inlineStr">
+      <c r="D198" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>4,940.4000</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
         <is>
           <t>4,940.4 au.  ด้านภัยพิบัต</t>
         </is>
@@ -7081,96 +7141,108 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" t="n">
+      <c r="A201" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B201" t="n">
+      <c r="B201" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="C201" t="inlineStr">
+      <c r="C201" s="2" t="inlineStr">
         <is>
           <t>115,694.0</t>
         </is>
       </c>
-      <c r="D201" t="n">
-        <v>1</v>
-      </c>
-      <c r="E201" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F201" t="inlineStr">
-        <is>
-          <t>115,694.0</t>
-        </is>
-      </c>
-      <c r="G201" t="inlineStr"/>
-      <c r="H201" t="inlineStr">
+      <c r="D201" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t>115,694.0000</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
         <is>
           <t>115,694.0 au. พัฒนาระบบประก</t>
         </is>
       </c>
     </row>
     <row r="202">
-      <c r="A202" t="n">
+      <c r="A202" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B202" t="n">
+      <c r="B202" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="C202" t="inlineStr">
+      <c r="C202" s="2" t="inlineStr">
         <is>
           <t>4,800.0</t>
         </is>
       </c>
-      <c r="D202" t="n">
-        <v>1</v>
-      </c>
-      <c r="E202" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F202" t="inlineStr">
-        <is>
-          <t>4,800.0</t>
-        </is>
-      </c>
-      <c r="G202" t="inlineStr"/>
-      <c r="H202" t="inlineStr">
+      <c r="D202" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>4,800.0000</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
         <is>
           <t>4,800.0 au. ผลักด้นให้ประ</t>
         </is>
       </c>
     </row>
     <row r="203">
-      <c r="A203" t="n">
+      <c r="A203" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B203" t="n">
+      <c r="B203" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="C203" t="inlineStr">
+      <c r="C203" s="2" t="inlineStr">
         <is>
           <t>44,492.1</t>
         </is>
       </c>
-      <c r="D203" t="n">
-        <v>1</v>
-      </c>
-      <c r="E203" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F203" t="inlineStr">
-        <is>
-          <t>44,492.1</t>
-        </is>
-      </c>
-      <c r="G203" t="inlineStr"/>
-      <c r="H203" t="inlineStr">
+      <c r="D203" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>44,492.1000</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
         <is>
           <t>44,492.1 au. การอนุรักษ์แล</t>
         </is>
@@ -7213,64 +7285,72 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" t="n">
+      <c r="A205" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B205" t="n">
+      <c r="B205" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="C205" t="inlineStr">
+      <c r="C205" s="2" t="inlineStr">
         <is>
           <t>25,537.2</t>
         </is>
       </c>
-      <c r="D205" t="n">
-        <v>1</v>
-      </c>
-      <c r="E205" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F205" t="inlineStr">
-        <is>
-          <t>25,537.2</t>
-        </is>
-      </c>
-      <c r="G205" t="inlineStr"/>
-      <c r="H205" t="inlineStr">
+      <c r="D205" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>25,537.2000</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="inlineStr">
         <is>
           <t>25,537.2 au.  การปฏิรูประบ</t>
         </is>
       </c>
     </row>
     <row r="206">
-      <c r="A206" t="n">
+      <c r="A206" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B206" t="n">
+      <c r="B206" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="C206" t="inlineStr">
+      <c r="C206" s="2" t="inlineStr">
         <is>
           <t>7,732.0</t>
         </is>
       </c>
-      <c r="D206" t="n">
-        <v>1</v>
-      </c>
-      <c r="E206" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F206" t="inlineStr">
-        <is>
-          <t>7,732.0</t>
-        </is>
-      </c>
-      <c r="G206" t="inlineStr"/>
-      <c r="H206" t="inlineStr">
+      <c r="D206" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>7,732.0000</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
         <is>
           <t>7,732.0 au.  การพัฒนากฎหม</t>
         </is>
@@ -7937,32 +8017,36 @@
       <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
-      <c r="A227" t="n">
+      <c r="A227" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B227" t="n">
+      <c r="B227" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="C227" t="inlineStr">
+      <c r="C227" s="2" t="inlineStr">
         <is>
           <t>709.5</t>
         </is>
       </c>
-      <c r="D227" t="n">
-        <v>1</v>
-      </c>
-      <c r="E227" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F227" t="inlineStr">
-        <is>
-          <t>709.5</t>
-        </is>
-      </c>
-      <c r="G227" t="inlineStr"/>
-      <c r="H227" t="inlineStr">
+      <c r="D227" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>709.5000</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H227" s="2" t="inlineStr">
         <is>
           <t>s:ui1du 709.5 auuain  BUDGET BU</t>
         </is>
@@ -8053,7 +8137,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
@@ -8249,7 +8333,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
@@ -8381,7 +8465,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -8477,7 +8561,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -8973,7 +9057,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -9473,7 +9557,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -9521,32 +9605,36 @@
       </c>
     </row>
     <row r="276">
-      <c r="A276" t="n">
+      <c r="A276" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="B276" t="n">
+      <c r="B276" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="C276" t="inlineStr">
+      <c r="C276" s="2" t="inlineStr">
         <is>
           <t>219,902.2</t>
         </is>
       </c>
-      <c r="D276" t="n">
-        <v>1</v>
-      </c>
-      <c r="E276" t="inlineStr">
-        <is>
-          <t>บาท (ต่อหน่วย)</t>
-        </is>
-      </c>
-      <c r="F276" t="inlineStr">
-        <is>
-          <t>219,902.2</t>
-        </is>
-      </c>
-      <c r="G276" t="inlineStr"/>
-      <c r="H276" t="inlineStr">
+      <c r="D276" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E276" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>219,902.2000</t>
+        </is>
+      </c>
+      <c r="G276" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H276" s="2" t="inlineStr">
         <is>
           <t>ป 219,902.2 ล่านบาท  เร่งจัดก</t>
         </is>
@@ -9569,7 +9657,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -9665,7 +9753,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -9793,7 +9881,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -9841,32 +9929,36 @@
       </c>
     </row>
     <row r="286">
-      <c r="A286" t="n">
+      <c r="A286" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="B286" t="n">
+      <c r="B286" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="C286" t="inlineStr">
+      <c r="C286" s="2" t="inlineStr">
         <is>
           <t>4,399</t>
         </is>
       </c>
-      <c r="D286" t="n">
-        <v>0</v>
-      </c>
-      <c r="E286" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F286" t="inlineStr">
-        <is>
-          <t>4,399</t>
-        </is>
-      </c>
-      <c r="G286" t="inlineStr"/>
-      <c r="H286" t="inlineStr">
+      <c r="D286" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>4,399.0000</t>
+        </is>
+      </c>
+      <c r="G286" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H286" s="2" t="inlineStr">
         <is>
           <t>้อยกว่า 4,399 au.  ผู้ประกอบการ</t>
         </is>
@@ -10169,32 +10261,36 @@
       </c>
     </row>
     <row r="296">
-      <c r="A296" t="n">
+      <c r="A296" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B296" t="n">
+      <c r="B296" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="C296" t="inlineStr">
+      <c r="C296" s="2" t="inlineStr">
         <is>
           <t>14,357.0</t>
         </is>
       </c>
-      <c r="D296" t="n">
-        <v>1</v>
-      </c>
-      <c r="E296" t="inlineStr">
-        <is>
-          <t>บาท (ต่อหน่วย)</t>
-        </is>
-      </c>
-      <c r="F296" t="inlineStr">
-        <is>
-          <t>14,357.0</t>
-        </is>
-      </c>
-      <c r="G296" t="inlineStr"/>
-      <c r="H296" t="inlineStr">
+      <c r="D296" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E296" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F296" s="2" t="inlineStr">
+        <is>
+          <t>14,357.0000</t>
+        </is>
+      </c>
+      <c r="G296" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H296" s="2" t="inlineStr">
         <is>
           <t>น”      14,357.0 ลานบาท  สร้างแรงอ</t>
         </is>
@@ -10249,7 +10345,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านไร่)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
@@ -10313,7 +10409,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านราย)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
@@ -10697,64 +10793,72 @@
       </c>
     </row>
     <row r="312">
-      <c r="A312" t="n">
+      <c r="A312" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="B312" t="n">
+      <c r="B312" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="C312" t="inlineStr">
+      <c r="C312" s="2" t="inlineStr">
         <is>
           <t>744.9</t>
         </is>
       </c>
-      <c r="D312" t="n">
-        <v>1</v>
-      </c>
-      <c r="E312" t="inlineStr">
-        <is>
-          <t>บาท (ต่อหน่วย)</t>
-        </is>
-      </c>
-      <c r="F312" t="inlineStr">
-        <is>
-          <t>744.9</t>
-        </is>
-      </c>
-      <c r="G312" t="inlineStr"/>
-      <c r="H312" t="inlineStr">
+      <c r="D312" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E312" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F312" s="2" t="inlineStr">
+        <is>
+          <t>744.9000</t>
+        </is>
+      </c>
+      <c r="G312" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H312" s="2" t="inlineStr">
         <is>
           <t>”       744.9 ลานบาท  : การขับเ</t>
         </is>
       </c>
     </row>
     <row r="313">
-      <c r="A313" t="n">
+      <c r="A313" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="B313" t="n">
+      <c r="B313" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="C313" t="inlineStr">
+      <c r="C313" s="2" t="inlineStr">
         <is>
           <t>19,845.2</t>
         </is>
       </c>
-      <c r="D313" t="n">
-        <v>1</v>
-      </c>
-      <c r="E313" t="inlineStr">
-        <is>
-          <t>บาท (ต่อหน่วย)</t>
-        </is>
-      </c>
-      <c r="F313" t="inlineStr">
-        <is>
-          <t>19,845.2</t>
-        </is>
-      </c>
-      <c r="G313" t="inlineStr"/>
-      <c r="H313" t="inlineStr">
+      <c r="D313" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E313" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F313" s="2" t="inlineStr">
+        <is>
+          <t>19,845.2000</t>
+        </is>
+      </c>
+      <c r="G313" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H313" s="2" t="inlineStr">
         <is>
           <t>อ 19,845.2 ล่านบาท  ปข้องกัน</t>
         </is>
@@ -11601,7 +11705,7 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านราย)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
@@ -12253,7 +12357,7 @@
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
@@ -12285,7 +12389,7 @@
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
@@ -12509,7 +12613,7 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
@@ -12765,7 +12869,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
@@ -12849,32 +12953,36 @@
       </c>
     </row>
     <row r="379">
-      <c r="A379" t="n">
+      <c r="A379" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="B379" t="n">
+      <c r="B379" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="C379" t="inlineStr">
+      <c r="C379" s="2" t="inlineStr">
         <is>
           <t>303,490</t>
         </is>
       </c>
-      <c r="D379" t="n">
-        <v>0</v>
-      </c>
-      <c r="E379" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F379" t="inlineStr">
-        <is>
-          <t>303,490</t>
-        </is>
-      </c>
-      <c r="G379" t="inlineStr"/>
-      <c r="H379" t="inlineStr">
+      <c r="D379" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E379" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F379" s="2" t="inlineStr">
+        <is>
+          <t>303,490.0000</t>
+        </is>
+      </c>
+      <c r="G379" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H379" s="2" t="inlineStr">
         <is>
           <t>ในชุมชน 303,490 au ได้รับการส่งเส</t>
         </is>
@@ -12993,7 +13101,7 @@
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านราย)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
@@ -14221,7 +14329,7 @@
       </c>
       <c r="E421" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านคน)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F421" t="inlineStr">
@@ -14317,7 +14425,7 @@
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านไร่)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F424" t="inlineStr">
@@ -14381,7 +14489,7 @@
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านไร่)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F426" t="inlineStr">
@@ -14477,7 +14585,7 @@
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านไร่)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
@@ -14797,7 +14905,7 @@
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>จำนวน (ล้านราย)</t>
+          <t>จำนวน (ล้านหน่วย)</t>
         </is>
       </c>
       <c r="F439" t="inlineStr">
@@ -14905,64 +15013,72 @@
       </c>
     </row>
     <row r="443">
-      <c r="A443" t="n">
+      <c r="A443" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="B443" t="n">
+      <c r="B443" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="C443" t="inlineStr">
+      <c r="C443" s="2" t="inlineStr">
         <is>
           <t>611,220</t>
         </is>
       </c>
-      <c r="D443" t="n">
-        <v>0</v>
-      </c>
-      <c r="E443" t="inlineStr">
-        <is>
-          <t>ไม่ทราบหน่วย</t>
-        </is>
-      </c>
-      <c r="F443" t="inlineStr">
-        <is>
-          <t>611,220</t>
-        </is>
-      </c>
-      <c r="G443" t="inlineStr"/>
-      <c r="H443" t="inlineStr">
+      <c r="D443" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E443" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F443" s="2" t="inlineStr">
+        <is>
+          <t>611,220.0000</t>
+        </is>
+      </c>
+      <c r="G443" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H443" s="2" t="inlineStr">
         <is>
           <t>้อยกว่า 611,220 au.  จากสินค้าและ</t>
         </is>
       </c>
     </row>
     <row r="444">
-      <c r="A444" t="n">
+      <c r="A444" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="B444" t="n">
+      <c r="B444" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="C444" t="inlineStr">
+      <c r="C444" s="2" t="inlineStr">
         <is>
           <t>2,517,700</t>
         </is>
       </c>
-      <c r="D444" t="n">
-        <v>0</v>
-      </c>
-      <c r="E444" t="inlineStr">
-        <is>
-          <t>จำนวน (นับ)</t>
-        </is>
-      </c>
-      <c r="F444" t="inlineStr">
-        <is>
-          <t>2,517,700</t>
-        </is>
-      </c>
-      <c r="G444" t="inlineStr"/>
-      <c r="H444" t="inlineStr">
+      <c r="D444" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E444" s="2" t="inlineStr">
+        <is>
+          <t>ล้านบาท</t>
+        </is>
+      </c>
+      <c r="F444" s="2" t="inlineStr">
+        <is>
+          <t>2,517,700.0000</t>
+        </is>
+      </c>
+      <c r="G444" s="2" t="inlineStr">
+        <is>
+          <t>ใช่</t>
+        </is>
+      </c>
+      <c r="H444" s="2" t="inlineStr">
         <is>
           <t>้อยกว่า 2,517,700 au. อากภาษีรายได้</t>
         </is>

</xml_diff>